<commit_message>
Final unified Arabic review: report (PDF via Chromium, validated DOCX), Arabic RTL register (127 rows), email draft; fix docx schema error
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PwvPj41jSev9ApGi3qLq4f
</commit_message>
<xml_diff>
--- a/pmu-admissions-audit/final_review/سجل_ملاحظات_صفحات_مكتب_القبول.xlsx
+++ b/pmu-admissions-audit/final_review/سجل_ملاحظات_صفحات_مكتب_القبول.xlsx
@@ -8441,7 +8441,7 @@
       </c>
       <c r="B6" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> home</t>
+          <t>الصفحة الرئيسية للجامعة</t>
         </is>
       </c>
       <c r="C6" s="21" t="inlineStr">
@@ -8463,7 +8463,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Study at PMU :: PMU :: Prince Mohammad Bin Fahd University</t>
+          <t>صفحة Study @ PMU (مكتب التسجيل)</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">

</xml_diff>